<commit_message>
update descr extensions 9fd1b329c067da154525675eebde55615383c792
</commit_message>
<xml_diff>
--- a/nr-uniformisation-descriptions/ig/StructureDefinition-fr-core-address-insee-code.xlsx
+++ b/nr-uniformisation-descriptions/ig/StructureDefinition-fr-core-address-insee-code.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-11T11:03:37+00:00</t>
+    <t>2025-02-11T12:08:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t>This extension adds the insee code (5 digits) to the address | Ajout du code insee (5 chiffres) à l'adresse postale</t>
+    <t>Extension d'ajout du code insee (5 chiffres) à l'adresse postale.
+This extension adds the insee code (5 digits) to the address</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>